<commit_message>
finish updateind 2.qmd, attempt recalculate gq pop
- inconsistent GQ pop at census tract level. Skipping for now.
</commit_message>
<xml_diff>
--- a/_Source - CollegeControlTotal - 2025-02-14_Start.xlsx
+++ b/_Source - CollegeControlTotal - 2025-02-14_Start.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Desktop_Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\TDM-INP-College-Enrollment\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E45F1F1-8399-4D09-8170-582139454AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="270" windowWidth="28800" windowHeight="14655" tabRatio="728" firstSheet="3" activeTab="9"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="728" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export_ControlTot" sheetId="11" r:id="rId1"/>
@@ -29,7 +30,7 @@
     <sheet name="USHE 2020 Campus Totals" sheetId="3" r:id="rId15"/>
     <sheet name="MAG College Enrollment Forecast" sheetId="12" r:id="rId16"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="201">
   <si>
     <t>https://ushe.edu/institutional-data-resources-headcount/</t>
   </si>
@@ -612,9 +613,6 @@
     <t>Source: 2019 RTP</t>
   </si>
   <si>
-    <t>Source: USHE Enrollment data by Zip (Base Distribution Jupyter Notebook)</t>
-  </si>
-  <si>
     <t>Note:</t>
   </si>
   <si>
@@ -659,11 +657,38 @@
   <si>
     <t>*USHE not currently releasing updates forecasts</t>
   </si>
+  <si>
+    <t>Source: USHE Enrollment data by Zip (Base Distribution: 4-CollegeCampusDisaggregation.Rmd)</t>
+  </si>
+  <si>
+    <t>Old Data</t>
+  </si>
+  <si>
+    <t>Might have to fill this.</t>
+  </si>
+  <si>
+    <t>Need to update</t>
+  </si>
+  <si>
+    <t>Probably from College Survey</t>
+  </si>
+  <si>
+    <t>Not updated</t>
+  </si>
+  <si>
+    <t>This has to update to 2055</t>
+  </si>
+  <si>
+    <t>project until 2060</t>
+  </si>
+  <si>
+    <t>Project until 2060</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
@@ -989,7 +1014,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1236,9 +1261,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1249,16 +1271,11 @@
     <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1268,7 +1285,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -1297,7 +1321,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1336,7 +1360,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1783,7 +1806,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -2200,7 +2223,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -2617,7 +2640,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -3034,7 +3057,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -3451,7 +3474,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -3868,7 +3891,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -4287,7 +4310,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -4706,7 +4729,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000007-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -5125,7 +5148,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000008-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -5544,7 +5567,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000009-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -5963,7 +5986,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{0000000A-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -6382,7 +6405,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{0000000B-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -6802,7 +6825,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{0000000C-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -7222,7 +7245,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{0000000D-6C95-4AF9-9677-75D0BF8DBF4A}"/>
             </c:ext>
@@ -7374,7 +7397,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -7407,7 +7429,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -7449,7 +7471,7 @@
 </file>
 
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -7623,7 +7645,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-F488-4F6F-B8FC-239954948267}"/>
             </c:ext>
@@ -7751,7 +7773,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-F488-4F6F-B8FC-239954948267}"/>
             </c:ext>
@@ -7810,7 +7832,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-F488-4F6F-B8FC-239954948267}"/>
             </c:ext>
@@ -8037,7 +8059,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-9DD6-48A5-BA59-1EDEEA739F36}"/>
             </c:ext>
@@ -8200,7 +8222,6 @@
         <c:idx val="5"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -8233,7 +8254,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -8275,7 +8296,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -8314,7 +8335,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -8761,7 +8781,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-7425-44AD-8193-F239116FDCF5}"/>
             </c:ext>
@@ -8914,7 +8934,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="zero"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -8956,7 +8976,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -8995,7 +9015,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -9262,7 +9281,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-54C9-4473-BE7D-5D3B04CD9771}"/>
             </c:ext>
@@ -9415,7 +9434,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="zero"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -9457,7 +9476,7 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -9736,7 +9755,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-1282-4053-85BF-D36622F55D0B}"/>
             </c:ext>
@@ -9840,7 +9859,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-1282-4053-85BF-D36622F55D0B}"/>
             </c:ext>
@@ -9968,7 +9987,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-1282-4053-85BF-D36622F55D0B}"/>
             </c:ext>
@@ -10027,7 +10046,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-1282-4053-85BF-D36622F55D0B}"/>
             </c:ext>
@@ -10212,7 +10231,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-5579-4878-B9E0-D9341EFE46CF}"/>
             </c:ext>
@@ -10378,7 +10397,6 @@
         <c:idx val="7"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -10411,7 +10429,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -10453,7 +10471,7 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -10732,7 +10750,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-437D-441E-8CA1-A3C31C8FEFD5}"/>
             </c:ext>
@@ -10836,7 +10854,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-437D-441E-8CA1-A3C31C8FEFD5}"/>
             </c:ext>
@@ -10964,7 +10982,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-437D-441E-8CA1-A3C31C8FEFD5}"/>
             </c:ext>
@@ -11023,7 +11041,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-437D-441E-8CA1-A3C31C8FEFD5}"/>
             </c:ext>
@@ -11206,7 +11224,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-8291-4C9C-9FB1-308A80325282}"/>
             </c:ext>
@@ -11372,7 +11390,6 @@
         <c:idx val="7"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -11405,7 +11422,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -11447,7 +11464,7 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -11726,7 +11743,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-262C-4D1B-BB8B-E4F7AB8B87B9}"/>
             </c:ext>
@@ -11830,7 +11847,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-262C-4D1B-BB8B-E4F7AB8B87B9}"/>
             </c:ext>
@@ -11958,7 +11975,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-262C-4D1B-BB8B-E4F7AB8B87B9}"/>
             </c:ext>
@@ -12017,7 +12034,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-262C-4D1B-BB8B-E4F7AB8B87B9}"/>
             </c:ext>
@@ -12069,7 +12086,7 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000004-7773-4901-91E0-F1EA12BDB5F6}"/>
               </c:ext>
@@ -12226,7 +12243,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-7773-4901-91E0-F1EA12BDB5F6}"/>
             </c:ext>
@@ -12391,7 +12408,6 @@
         <c:idx val="7"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -12424,7 +12440,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -12466,7 +12482,7 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -12745,7 +12761,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-B831-4F91-A79F-255456EFB6C8}"/>
             </c:ext>
@@ -12849,7 +12865,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-B831-4F91-A79F-255456EFB6C8}"/>
             </c:ext>
@@ -12977,7 +12993,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-B831-4F91-A79F-255456EFB6C8}"/>
             </c:ext>
@@ -13029,7 +13045,7 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-94A6-487E-A6F0-693E2BB8A9D8}"/>
               </c:ext>
@@ -13060,7 +13076,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-B831-4F91-A79F-255456EFB6C8}"/>
             </c:ext>
@@ -13245,7 +13261,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-94A6-487E-A6F0-693E2BB8A9D8}"/>
             </c:ext>
@@ -13410,7 +13426,6 @@
         <c:idx val="7"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -13443,7 +13458,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -13485,7 +13500,7 @@
 </file>
 
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -13800,7 +13815,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-3A74-4781-ACED-B1A98497F406}"/>
             </c:ext>
@@ -13928,7 +13943,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000005-3A74-4781-ACED-B1A98497F406}"/>
             </c:ext>
@@ -13987,7 +14002,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-3A74-4781-ACED-B1A98497F406}"/>
             </c:ext>
@@ -14172,7 +14187,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-C237-4535-B7C7-31175CD4A089}"/>
             </c:ext>
@@ -14334,7 +14349,6 @@
         <c:idx val="5"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -14367,7 +14381,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -14409,7 +14423,7 @@
 </file>
 
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -14631,7 +14645,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-BC61-47BB-8BCF-8D1D611131B5}"/>
             </c:ext>
@@ -14759,7 +14773,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000007-BC61-47BB-8BCF-8D1D611131B5}"/>
             </c:ext>
@@ -14818,7 +14832,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000006-BC61-47BB-8BCF-8D1D611131B5}"/>
             </c:ext>
@@ -15057,7 +15071,7 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-330F-41CF-8E17-74E90AC63C64}"/>
             </c:ext>
@@ -15220,7 +15234,6 @@
         <c:idx val="5"/>
         <c:delete val="1"/>
       </c:legendEntry>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -15253,7 +15266,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+    <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
@@ -20861,7 +20874,7 @@
         <xdr:cNvPr id="5" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{C758BB74-C52F-4EAC-94E7-B3D4F20B9207}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C758BB74-C52F-4EAC-94E7-B3D4F20B9207}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -20899,7 +20912,7 @@
         <xdr:cNvPr id="6" name="Chart 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{C94BF622-72F0-4EFA-BC03-32D40E0BBD94}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C94BF622-72F0-4EFA-BC03-32D40E0BBD94}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -20937,7 +20950,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{3BBA52D3-63EA-4037-953A-D61CA982A75E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3BBA52D3-63EA-4037-953A-D61CA982A75E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -20980,7 +20993,7 @@
         <xdr:cNvPr id="22" name="Chart 21">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{91CBB898-A0E3-4288-BDC2-BBC243FF9881}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{91CBB898-A0E3-4288-BDC2-BBC243FF9881}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21018,7 +21031,7 @@
         <xdr:cNvPr id="23" name="Chart 22">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{986BAAD4-A38A-44BC-9BB3-A50EF5713D36}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{986BAAD4-A38A-44BC-9BB3-A50EF5713D36}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21056,7 +21069,7 @@
         <xdr:cNvPr id="24" name="Chart 23">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{C722CC9E-91F6-4CCE-B1CA-D400ED437365}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C722CC9E-91F6-4CCE-B1CA-D400ED437365}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21094,7 +21107,7 @@
         <xdr:cNvPr id="25" name="Chart 24">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{E654136D-6A0F-48C7-956E-AB3F5802EF67}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E654136D-6A0F-48C7-956E-AB3F5802EF67}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21132,7 +21145,7 @@
         <xdr:cNvPr id="26" name="Chart 25">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{4A8DC08F-17BB-4ABD-BD3A-683405BC91AE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A8DC08F-17BB-4ABD-BD3A-683405BC91AE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21170,7 +21183,7 @@
         <xdr:cNvPr id="27" name="Chart 26">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{EDD82B92-0E97-430E-B1C0-7360767BC560}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDD82B92-0E97-430E-B1C0-7360767BC560}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21208,7 +21221,7 @@
         <xdr:cNvPr id="28" name="Chart 27">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{BD3D5500-528B-4495-824B-EA310EF9350E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD3D5500-528B-4495-824B-EA310EF9350E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21251,7 +21264,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{47530349-986F-478B-A6D0-1E72A1F89A82}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47530349-986F-478B-A6D0-1E72A1F89A82}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21300,7 +21313,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{4531E8D3-0968-B75F-63E7-FF06CB98CD51}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4531E8D3-0968-B75F-63E7-FF06CB98CD51}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21344,7 +21357,7 @@
         <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{8FA0C9D7-0378-F096-6D5D-527CEC9544E7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8FA0C9D7-0378-F096-6D5D-527CEC9544E7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21393,7 +21406,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{0781F624-165D-C4E0-0E48-2671E8E54B1B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0781F624-165D-C4E0-0E48-2671E8E54B1B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21437,7 +21450,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{5A6F2C61-FDAA-4F11-AF09-896FF347EA9E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A6F2C61-FDAA-4F11-AF09-896FF347EA9E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21481,7 +21494,7 @@
         <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A88477F1-82C0-4588-9DC9-0A2ACFCF53A5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A88477F1-82C0-4588-9DC9-0A2ACFCF53A5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21522,7 +21535,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4"/>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0B00-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -21568,7 +21587,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{1669A7C5-91D1-386D-B34B-63981ED3867C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1669A7C5-91D1-386D-B34B-63981ED3867C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21612,7 +21631,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{C8870E41-0605-E35C-E6EA-37BDB88F8961}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8870E41-0605-E35C-E6EA-37BDB88F8961}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21656,7 +21675,7 @@
         <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{98490862-385D-1115-23E8-5ED696D2B097}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98490862-385D-1115-23E8-5ED696D2B097}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21700,7 +21719,7 @@
         <xdr:cNvPr id="7" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{34C79F7D-5658-8BC3-7BC4-72F2AA87B54A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34C79F7D-5658-8BC3-7BC4-72F2AA87B54A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21744,7 +21763,7 @@
         <xdr:cNvPr id="8" name="Picture 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{FF116E29-9E89-1CF2-8D49-C419987E21F5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF116E29-9E89-1CF2-8D49-C419987E21F5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21788,7 +21807,7 @@
         <xdr:cNvPr id="9" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00A210A5-1DBD-D610-610B-69C854F5301C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00A210A5-1DBD-D610-610B-69C854F5301C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -21829,7 +21848,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4"/>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0C00-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -21867,7 +21892,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 9"/>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0C00-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -21905,7 +21936,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Picture 10"/>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0C00-00000B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -21943,7 +21980,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11"/>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0C00-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -22265,11 +22308,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:U62"/>
+  <dimension ref="A1:U73"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="15" width="12.140625" style="7" customWidth="1"/>
@@ -26045,6 +26088,62 @@
         <v>3000</v>
       </c>
     </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A63" s="7">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A64" s="7">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="7">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="7">
+        <v>2054</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="7">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="7">
+        <v>2056</v>
+      </c>
+      <c r="B68" s="108"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="7">
+        <v>2057</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="7">
+        <v>2058</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="7">
+        <v>2059</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="7">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="109" t="s">
+        <v>198</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -26052,7 +26151,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -26078,30 +26177,30 @@
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="J2" s="5"/>
-      <c r="Q2" s="105" t="s">
+      <c r="Q2" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="106"/>
-      <c r="S2" s="106"/>
-      <c r="T2" s="106"/>
-      <c r="U2" s="105" t="s">
+      <c r="R2" s="104"/>
+      <c r="S2" s="104"/>
+      <c r="T2" s="104"/>
+      <c r="U2" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="106"/>
-      <c r="W2" s="106"/>
-      <c r="X2" s="106"/>
-      <c r="Y2" s="105" t="s">
+      <c r="V2" s="104"/>
+      <c r="W2" s="104"/>
+      <c r="X2" s="104"/>
+      <c r="Y2" s="103" t="s">
         <v>3</v>
       </c>
-      <c r="Z2" s="106"/>
-      <c r="AA2" s="106"/>
-      <c r="AB2" s="106"/>
-      <c r="AC2" s="105" t="s">
+      <c r="Z2" s="104"/>
+      <c r="AA2" s="104"/>
+      <c r="AB2" s="104"/>
+      <c r="AC2" s="103" t="s">
         <v>4</v>
       </c>
-      <c r="AD2" s="106"/>
-      <c r="AE2" s="106"/>
-      <c r="AF2" s="106"/>
+      <c r="AD2" s="104"/>
+      <c r="AE2" s="104"/>
+      <c r="AF2" s="104"/>
     </row>
     <row r="3" spans="1:32" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -26757,12 +26856,12 @@
       <c r="AC10" s="43">
         <v>5812</v>
       </c>
-      <c r="AD10" s="104"/>
-      <c r="AE10" s="104"/>
-      <c r="AF10" s="104"/>
+      <c r="AD10" s="44"/>
+      <c r="AE10" s="44"/>
+      <c r="AF10" s="44"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A11" s="96">
+      <c r="A11" s="3">
         <v>2023</v>
       </c>
       <c r="B11" s="18">
@@ -26786,7 +26885,7 @@
       <c r="H11" s="18">
         <v>6369</v>
       </c>
-      <c r="J11" s="96">
+      <c r="J11" s="3">
         <v>2023</v>
       </c>
       <c r="K11" s="26">
@@ -26805,7 +26904,7 @@
         <f t="shared" si="3"/>
         <v>5949</v>
       </c>
-      <c r="P11" s="103">
+      <c r="P11" s="101">
         <v>2023</v>
       </c>
       <c r="Q11" s="43">
@@ -26845,12 +26944,12 @@
       <c r="AC11" s="43">
         <v>5949</v>
       </c>
-      <c r="AD11" s="104"/>
-      <c r="AE11" s="104"/>
-      <c r="AF11" s="104"/>
+      <c r="AD11" s="44"/>
+      <c r="AE11" s="44"/>
+      <c r="AF11" s="44"/>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A12" s="96">
+      <c r="A12" s="3">
         <v>2024</v>
       </c>
       <c r="B12" s="18">
@@ -26865,7 +26964,7 @@
       <c r="E12" s="18">
         <v>27437</v>
       </c>
-      <c r="J12" s="96">
+      <c r="J12" s="3">
         <v>2024</v>
       </c>
       <c r="K12" s="26">
@@ -26884,7 +26983,7 @@
         <f t="shared" si="3"/>
         <v>6142</v>
       </c>
-      <c r="P12" s="103">
+      <c r="P12" s="101">
         <v>2024</v>
       </c>
       <c r="Q12" s="43">
@@ -26924,9 +27023,14 @@
       <c r="AC12" s="43">
         <v>6142</v>
       </c>
-      <c r="AD12" s="104"/>
-      <c r="AE12" s="104"/>
-      <c r="AF12" s="104"/>
+      <c r="AD12" s="44"/>
+      <c r="AE12" s="44"/>
+      <c r="AF12" s="44"/>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="F13" s="42" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
@@ -26966,11 +27070,11 @@
     <mergeCell ref="AC2:AF2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B19" r:id="rId1"/>
-    <hyperlink ref="B18" r:id="rId2"/>
-    <hyperlink ref="P19" r:id="rId3"/>
-    <hyperlink ref="B17" r:id="rId4"/>
-    <hyperlink ref="B16" r:id="rId5"/>
+    <hyperlink ref="B19" r:id="rId1" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
+    <hyperlink ref="B18" r:id="rId2" xr:uid="{00000000-0004-0000-0900-000001000000}"/>
+    <hyperlink ref="P19" r:id="rId3" xr:uid="{00000000-0004-0000-0900-000002000000}"/>
+    <hyperlink ref="B17" r:id="rId4" xr:uid="{00000000-0004-0000-0900-000003000000}"/>
+    <hyperlink ref="B16" r:id="rId5" xr:uid="{00000000-0004-0000-0900-000004000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId6"/>
@@ -26979,7 +27083,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -27030,13 +27134,13 @@
         <v>81</v>
       </c>
       <c r="L1" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="N1" s="16" t="s">
         <v>182</v>
-      </c>
-      <c r="N1" s="16" t="s">
-        <v>183</v>
       </c>
       <c r="O1" s="16" t="s">
         <v>80</v>
@@ -27066,13 +27170,13 @@
         <v>72</v>
       </c>
       <c r="X1" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="Y1" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="Y1" s="16" t="s">
+      <c r="Z1" s="16" t="s">
         <v>187</v>
-      </c>
-      <c r="Z1" s="16" t="s">
-        <v>188</v>
       </c>
       <c r="AA1" s="16" t="s">
         <v>71</v>
@@ -27102,13 +27206,13 @@
         <v>63</v>
       </c>
       <c r="AJ1" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="AK1" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="AK1" s="16" t="s">
+      <c r="AL1" s="16" t="s">
         <v>190</v>
-      </c>
-      <c r="AL1" s="16" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.25">
@@ -27448,15 +27552,15 @@
     </row>
     <row r="8" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>185</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B8" r:id="rId1" location="enrollment"/>
+    <hyperlink ref="B8" r:id="rId1" location="enrollment" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId2"/>
@@ -27464,7 +27568,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -27529,7 +27633,7 @@
       <c r="N3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="102">
+      <c r="V3" s="100">
         <v>45702</v>
       </c>
     </row>
@@ -27772,7 +27876,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="96">
+      <c r="A18" s="3">
         <v>2022</v>
       </c>
       <c r="B18" s="33">
@@ -27786,7 +27890,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="96">
+      <c r="A19" s="3">
         <v>2023</v>
       </c>
       <c r="B19" s="33">
@@ -27800,7 +27904,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="96">
+      <c r="A20" s="3">
         <v>2024</v>
       </c>
       <c r="B20" s="33">
@@ -27815,8 +27919,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="N3" r:id="rId2"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{00000000-0004-0000-0B00-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>
@@ -27825,7 +27929,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -27896,6 +28000,15 @@
         <v>1929</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>2020</v>
+      </c>
+      <c r="B8" s="106">
+        <f>AVERAGE(B7,B9)</f>
+        <v>1830</v>
+      </c>
+    </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="41">
         <v>2021</v>
@@ -27930,7 +28043,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D1" r:id="rId1"/>
+    <hyperlink ref="D1" r:id="rId1" xr:uid="{00000000-0004-0000-0C00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
@@ -27938,7 +28051,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -29404,7 +29517,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -29436,7 +29549,7 @@
         <v>50</v>
       </c>
       <c r="F1" s="95" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
@@ -29454,6 +29567,9 @@
       <c r="E2" s="12">
         <v>6</v>
       </c>
+      <c r="F2" s="42" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
@@ -29888,196 +30004,196 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="107" t="s">
+      <c r="B31" s="105" t="s">
         <v>46</v>
       </c>
-      <c r="C31" s="107"/>
-      <c r="D31" s="107"/>
-      <c r="E31" s="107"/>
+      <c r="C31" s="105"/>
+      <c r="D31" s="105"/>
+      <c r="E31" s="105"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="107"/>
-      <c r="C32" s="107"/>
-      <c r="D32" s="107"/>
-      <c r="E32" s="107"/>
+      <c r="B32" s="105"/>
+      <c r="C32" s="105"/>
+      <c r="D32" s="105"/>
+      <c r="E32" s="105"/>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="107"/>
-      <c r="C33" s="107"/>
-      <c r="D33" s="107"/>
-      <c r="E33" s="107"/>
+      <c r="B33" s="105"/>
+      <c r="C33" s="105"/>
+      <c r="D33" s="105"/>
+      <c r="E33" s="105"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" s="107"/>
-      <c r="C34" s="107"/>
-      <c r="D34" s="107"/>
-      <c r="E34" s="107"/>
+      <c r="B34" s="105"/>
+      <c r="C34" s="105"/>
+      <c r="D34" s="105"/>
+      <c r="E34" s="105"/>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="107"/>
-      <c r="C35" s="107"/>
-      <c r="D35" s="107"/>
-      <c r="E35" s="107"/>
+      <c r="B35" s="105"/>
+      <c r="C35" s="105"/>
+      <c r="D35" s="105"/>
+      <c r="E35" s="105"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B36" s="107"/>
-      <c r="C36" s="107"/>
-      <c r="D36" s="107"/>
-      <c r="E36" s="107"/>
+      <c r="B36" s="105"/>
+      <c r="C36" s="105"/>
+      <c r="D36" s="105"/>
+      <c r="E36" s="105"/>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B37" s="107"/>
-      <c r="C37" s="107"/>
-      <c r="D37" s="107"/>
-      <c r="E37" s="107"/>
+      <c r="B37" s="105"/>
+      <c r="C37" s="105"/>
+      <c r="D37" s="105"/>
+      <c r="E37" s="105"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B38" s="107"/>
-      <c r="C38" s="107"/>
-      <c r="D38" s="107"/>
-      <c r="E38" s="107"/>
+      <c r="B38" s="105"/>
+      <c r="C38" s="105"/>
+      <c r="D38" s="105"/>
+      <c r="E38" s="105"/>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B39" s="107"/>
-      <c r="C39" s="107"/>
-      <c r="D39" s="107"/>
-      <c r="E39" s="107"/>
+      <c r="B39" s="105"/>
+      <c r="C39" s="105"/>
+      <c r="D39" s="105"/>
+      <c r="E39" s="105"/>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B40" s="107"/>
-      <c r="C40" s="107"/>
-      <c r="D40" s="107"/>
-      <c r="E40" s="107"/>
+      <c r="B40" s="105"/>
+      <c r="C40" s="105"/>
+      <c r="D40" s="105"/>
+      <c r="E40" s="105"/>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B41" s="107"/>
-      <c r="C41" s="107"/>
-      <c r="D41" s="107"/>
-      <c r="E41" s="107"/>
+      <c r="B41" s="105"/>
+      <c r="C41" s="105"/>
+      <c r="D41" s="105"/>
+      <c r="E41" s="105"/>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B42" s="107"/>
-      <c r="C42" s="107"/>
-      <c r="D42" s="107"/>
-      <c r="E42" s="107"/>
+      <c r="B42" s="105"/>
+      <c r="C42" s="105"/>
+      <c r="D42" s="105"/>
+      <c r="E42" s="105"/>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B43" s="107"/>
-      <c r="C43" s="107"/>
-      <c r="D43" s="107"/>
-      <c r="E43" s="107"/>
+      <c r="B43" s="105"/>
+      <c r="C43" s="105"/>
+      <c r="D43" s="105"/>
+      <c r="E43" s="105"/>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B44" s="107"/>
-      <c r="C44" s="107"/>
-      <c r="D44" s="107"/>
-      <c r="E44" s="107"/>
+      <c r="B44" s="105"/>
+      <c r="C44" s="105"/>
+      <c r="D44" s="105"/>
+      <c r="E44" s="105"/>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B46" s="107" t="s">
+      <c r="B46" s="105" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="107"/>
-      <c r="D46" s="107"/>
-      <c r="E46" s="107"/>
+      <c r="C46" s="105"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="105"/>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B47" s="107" t="s">
+      <c r="B47" s="105" t="s">
         <v>45</v>
       </c>
-      <c r="C47" s="107"/>
-      <c r="D47" s="107"/>
-      <c r="E47" s="107"/>
+      <c r="C47" s="105"/>
+      <c r="D47" s="105"/>
+      <c r="E47" s="105"/>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B48" s="107"/>
-      <c r="C48" s="107"/>
-      <c r="D48" s="107"/>
-      <c r="E48" s="107"/>
+      <c r="B48" s="105"/>
+      <c r="C48" s="105"/>
+      <c r="D48" s="105"/>
+      <c r="E48" s="105"/>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B49" s="107"/>
-      <c r="C49" s="107"/>
-      <c r="D49" s="107"/>
-      <c r="E49" s="107"/>
+      <c r="B49" s="105"/>
+      <c r="C49" s="105"/>
+      <c r="D49" s="105"/>
+      <c r="E49" s="105"/>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B50" s="107"/>
-      <c r="C50" s="107"/>
-      <c r="D50" s="107"/>
-      <c r="E50" s="107"/>
+      <c r="B50" s="105"/>
+      <c r="C50" s="105"/>
+      <c r="D50" s="105"/>
+      <c r="E50" s="105"/>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B51" s="107"/>
-      <c r="C51" s="107"/>
-      <c r="D51" s="107"/>
-      <c r="E51" s="107"/>
+      <c r="B51" s="105"/>
+      <c r="C51" s="105"/>
+      <c r="D51" s="105"/>
+      <c r="E51" s="105"/>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B52" s="107"/>
-      <c r="C52" s="107"/>
-      <c r="D52" s="107"/>
-      <c r="E52" s="107"/>
+      <c r="B52" s="105"/>
+      <c r="C52" s="105"/>
+      <c r="D52" s="105"/>
+      <c r="E52" s="105"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B53" s="107"/>
-      <c r="C53" s="107"/>
-      <c r="D53" s="107"/>
-      <c r="E53" s="107"/>
+      <c r="B53" s="105"/>
+      <c r="C53" s="105"/>
+      <c r="D53" s="105"/>
+      <c r="E53" s="105"/>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B54" s="107"/>
-      <c r="C54" s="107"/>
-      <c r="D54" s="107"/>
-      <c r="E54" s="107"/>
+      <c r="B54" s="105"/>
+      <c r="C54" s="105"/>
+      <c r="D54" s="105"/>
+      <c r="E54" s="105"/>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B55" s="107"/>
-      <c r="C55" s="107"/>
-      <c r="D55" s="107"/>
-      <c r="E55" s="107"/>
+      <c r="B55" s="105"/>
+      <c r="C55" s="105"/>
+      <c r="D55" s="105"/>
+      <c r="E55" s="105"/>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B56" s="107"/>
-      <c r="C56" s="107"/>
-      <c r="D56" s="107"/>
-      <c r="E56" s="107"/>
+      <c r="B56" s="105"/>
+      <c r="C56" s="105"/>
+      <c r="D56" s="105"/>
+      <c r="E56" s="105"/>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B57" s="107"/>
-      <c r="C57" s="107"/>
-      <c r="D57" s="107"/>
-      <c r="E57" s="107"/>
+      <c r="B57" s="105"/>
+      <c r="C57" s="105"/>
+      <c r="D57" s="105"/>
+      <c r="E57" s="105"/>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B58" s="107"/>
-      <c r="C58" s="107"/>
-      <c r="D58" s="107"/>
-      <c r="E58" s="107"/>
+      <c r="B58" s="105"/>
+      <c r="C58" s="105"/>
+      <c r="D58" s="105"/>
+      <c r="E58" s="105"/>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B59" s="107"/>
-      <c r="C59" s="107"/>
-      <c r="D59" s="107"/>
-      <c r="E59" s="107"/>
+      <c r="B59" s="105"/>
+      <c r="C59" s="105"/>
+      <c r="D59" s="105"/>
+      <c r="E59" s="105"/>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B60" s="107"/>
-      <c r="C60" s="107"/>
-      <c r="D60" s="107"/>
-      <c r="E60" s="107"/>
+      <c r="B60" s="105"/>
+      <c r="C60" s="105"/>
+      <c r="D60" s="105"/>
+      <c r="E60" s="105"/>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B61" s="107"/>
-      <c r="C61" s="107"/>
-      <c r="D61" s="107"/>
-      <c r="E61" s="107"/>
+      <c r="B61" s="105"/>
+      <c r="C61" s="105"/>
+      <c r="D61" s="105"/>
+      <c r="E61" s="105"/>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B62" s="107"/>
-      <c r="C62" s="107"/>
-      <c r="D62" s="107"/>
-      <c r="E62" s="107"/>
+      <c r="B62" s="105"/>
+      <c r="C62" s="105"/>
+      <c r="D62" s="105"/>
+      <c r="E62" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -30089,7 +30205,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -31764,7 +31880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
@@ -31778,43 +31894,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="96" t="s">
         <v>175</v>
       </c>
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="97" t="s">
+      <c r="C1" s="96" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="97" t="s">
+      <c r="D1" s="96" t="s">
         <v>100</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="97" t="s">
+      <c r="F1" s="96" t="s">
         <v>107</v>
       </c>
-      <c r="G1" s="97" t="s">
+      <c r="G1" s="96" t="s">
         <v>106</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="I1" s="97" t="s">
+      <c r="I1" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="J1" s="97" t="s">
+      <c r="J1" s="96" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="97" t="s">
+      <c r="K1" s="96" t="s">
         <v>53</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="M1" s="97" t="s">
+      <c r="M1" s="96" t="s">
         <v>54</v>
       </c>
       <c r="N1" s="3" t="s">
@@ -31832,22 +31948,22 @@
       <c r="R1" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="S1" s="97" t="s">
+      <c r="S1" s="96" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="97" t="s">
+      <c r="T1" s="96" t="s">
         <v>101</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="V1" s="97" t="s">
+      <c r="V1" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="W1" s="97" t="s">
+      <c r="W1" s="96" t="s">
         <v>123</v>
       </c>
-      <c r="X1" s="97" t="s">
+      <c r="X1" s="96" t="s">
         <v>122</v>
       </c>
       <c r="Y1" s="3" t="s">
@@ -31870,7 +31986,7 @@
         <f>VLOOKUP(D1,'calc%concurrent'!$A$2:$B$15,2,FALSE)</f>
         <v>2.6040514489776623E-2</v>
       </c>
-      <c r="E2" s="100">
+      <c r="E2" s="99">
         <f>D2</f>
         <v>2.6040514489776623E-2</v>
       </c>
@@ -31882,7 +31998,7 @@
         <f>VLOOKUP(G1,'calc%concurrent'!$A$2:$B$15,2,FALSE)</f>
         <v>0.30851477449455678</v>
       </c>
-      <c r="H2" s="100">
+      <c r="H2" s="99">
         <f>G2</f>
         <v>0.30851477449455678</v>
       </c>
@@ -31898,7 +32014,7 @@
         <f>VLOOKUP(K1,'calc%concurrent'!$A$2:$B$15,2,FALSE)</f>
         <v>0.34092450566077115</v>
       </c>
-      <c r="L2" s="100">
+      <c r="L2" s="99">
         <f>K2</f>
         <v>0.34092450566077115</v>
       </c>
@@ -31906,23 +32022,23 @@
         <f>VLOOKUP(M1,'calc%concurrent'!$A$2:$B$15,2,FALSE)</f>
         <v>0.34092450566077115</v>
       </c>
-      <c r="N2" s="100">
+      <c r="N2" s="99">
         <f t="shared" ref="N2:R4" si="0">M2</f>
         <v>0.34092450566077115</v>
       </c>
-      <c r="O2" s="100">
+      <c r="O2" s="99">
         <f t="shared" si="0"/>
         <v>0.34092450566077115</v>
       </c>
-      <c r="P2" s="100">
+      <c r="P2" s="99">
         <f t="shared" si="0"/>
         <v>0.34092450566077115</v>
       </c>
-      <c r="Q2" s="100">
+      <c r="Q2" s="99">
         <f t="shared" si="0"/>
         <v>0.34092450566077115</v>
       </c>
-      <c r="R2" s="100">
+      <c r="R2" s="99">
         <f t="shared" si="0"/>
         <v>0.34092450566077115</v>
       </c>
@@ -31934,7 +32050,7 @@
         <f>VLOOKUP(T1,'calc%concurrent'!$A$2:$B$15,2,FALSE)</f>
         <v>0.26992028734364659</v>
       </c>
-      <c r="U2" s="100">
+      <c r="U2" s="99">
         <f>T2</f>
         <v>0.26992028734364659</v>
       </c>
@@ -31970,7 +32086,7 @@
         <f>VLOOKUP(D$1,'FTE Rate Calcs'!$A$2:$B$15,2,FALSE)</f>
         <v>1.0252202452927968</v>
       </c>
-      <c r="E3" s="100">
+      <c r="E3" s="99">
         <f t="shared" ref="E3:E4" si="1">D3</f>
         <v>1.0252202452927968</v>
       </c>
@@ -31982,7 +32098,7 @@
         <f>VLOOKUP(G$1,'FTE Rate Calcs'!$A$2:$B$15,2,FALSE)</f>
         <v>1.0375684282085227</v>
       </c>
-      <c r="H3" s="100">
+      <c r="H3" s="99">
         <f t="shared" ref="H3:H4" si="2">G3</f>
         <v>1.0375684282085227</v>
       </c>
@@ -31998,7 +32114,7 @@
         <f>VLOOKUP(K$1,'FTE Rate Calcs'!$A$2:$B$15,2,FALSE)</f>
         <v>1.2081372400182178</v>
       </c>
-      <c r="L3" s="100">
+      <c r="L3" s="99">
         <f t="shared" ref="L3:L4" si="3">K3</f>
         <v>1.2081372400182178</v>
       </c>
@@ -32006,23 +32122,23 @@
         <f>VLOOKUP(M$1,'FTE Rate Calcs'!$A$2:$B$15,2,FALSE)</f>
         <v>1.2081372400182178</v>
       </c>
-      <c r="N3" s="100">
+      <c r="N3" s="99">
         <f t="shared" si="0"/>
         <v>1.2081372400182178</v>
       </c>
-      <c r="O3" s="100">
+      <c r="O3" s="99">
         <f t="shared" si="0"/>
         <v>1.2081372400182178</v>
       </c>
-      <c r="P3" s="100">
+      <c r="P3" s="99">
         <f t="shared" si="0"/>
         <v>1.2081372400182178</v>
       </c>
-      <c r="Q3" s="100">
+      <c r="Q3" s="99">
         <f t="shared" si="0"/>
         <v>1.2081372400182178</v>
       </c>
-      <c r="R3" s="100">
+      <c r="R3" s="99">
         <f t="shared" si="0"/>
         <v>1.2081372400182178</v>
       </c>
@@ -32034,7 +32150,7 @@
         <f>VLOOKUP(T$1,'FTE Rate Calcs'!$A$2:$B$15,2,FALSE)</f>
         <v>1.0967771874057404</v>
       </c>
-      <c r="U3" s="100">
+      <c r="U3" s="99">
         <f t="shared" ref="U3:U4" si="4">T3</f>
         <v>1.0967771874057404</v>
       </c>
@@ -32070,7 +32186,7 @@
         <f>VLOOKUP(D$1,'HBC Rates'!$A$2:$B$15,2,FALSE)</f>
         <v>0.93010000000000004</v>
       </c>
-      <c r="E4" s="100">
+      <c r="E4" s="99">
         <f t="shared" si="1"/>
         <v>0.93010000000000004</v>
       </c>
@@ -32082,7 +32198,7 @@
         <f>VLOOKUP(G$1,'HBC Rates'!$A$2:$B$15,2,FALSE)</f>
         <v>0.67700000000000005</v>
       </c>
-      <c r="H4" s="100">
+      <c r="H4" s="99">
         <f t="shared" si="2"/>
         <v>0.67700000000000005</v>
       </c>
@@ -32098,7 +32214,7 @@
         <f>VLOOKUP(K$1,'HBC Rates'!$A$2:$B$15,2,FALSE)</f>
         <v>0.56869999999999998</v>
       </c>
-      <c r="L4" s="100">
+      <c r="L4" s="99">
         <f t="shared" si="3"/>
         <v>0.56869999999999998</v>
       </c>
@@ -32106,23 +32222,23 @@
         <f>VLOOKUP(M$1,'HBC Rates'!$A$2:$B$15,2,FALSE)</f>
         <v>0.61580000000000001</v>
       </c>
-      <c r="N4" s="100">
+      <c r="N4" s="99">
         <f t="shared" si="0"/>
         <v>0.61580000000000001</v>
       </c>
-      <c r="O4" s="100">
+      <c r="O4" s="99">
         <f t="shared" si="0"/>
         <v>0.61580000000000001</v>
       </c>
-      <c r="P4" s="100">
+      <c r="P4" s="99">
         <f t="shared" si="0"/>
         <v>0.61580000000000001</v>
       </c>
-      <c r="Q4" s="100">
+      <c r="Q4" s="99">
         <f t="shared" si="0"/>
         <v>0.61580000000000001</v>
       </c>
-      <c r="R4" s="100">
+      <c r="R4" s="99">
         <f t="shared" si="0"/>
         <v>0.61580000000000001</v>
       </c>
@@ -32134,7 +32250,7 @@
         <f>VLOOKUP(T$1,'HBC Rates'!$A$2:$B$15,2,FALSE)</f>
         <v>0.94520000000000004</v>
       </c>
-      <c r="U4" s="100">
+      <c r="U4" s="99">
         <f t="shared" si="4"/>
         <v>0.94520000000000004</v>
       </c>
@@ -32155,18 +32271,18 @@
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="98" t="s">
+      <c r="A6" s="97" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="98" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="99" t="s">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A8" s="98" t="s">
         <v>179</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="99" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
@@ -32180,8 +32296,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="O1:AQ65"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="O1:AQ66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="12" width="9" style="2"/>
@@ -36310,6 +36426,11 @@
         <v>241800</v>
       </c>
     </row>
+    <row r="66" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="O66" s="108" t="s">
+        <v>199</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -36318,12 +36439,13 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AZ64"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:AZ65"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="34" width="9" style="2"/>
-    <col min="35" max="42" width="9" style="7"/>
+    <col min="35" max="41" width="9" style="7"/>
+    <col min="42" max="42" width="10.42578125" style="7" customWidth="1"/>
     <col min="43" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -38705,6 +38827,11 @@
         <v>17</v>
       </c>
     </row>
+    <row r="65" spans="35:35" x14ac:dyDescent="0.25">
+      <c r="AI65" s="108" t="s">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -38713,7 +38840,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:T15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -39185,7 +39312,7 @@
         <f>$G$8</f>
         <v>1.0967771874057404</v>
       </c>
-      <c r="D9" s="101">
+      <c r="D9" s="3">
         <f t="shared" si="4"/>
         <v>2023</v>
       </c>
@@ -39193,14 +39320,14 @@
       <c r="F9" s="45"/>
       <c r="G9" s="45"/>
       <c r="H9" s="45"/>
-      <c r="J9" s="101">
+      <c r="J9" s="3">
         <v>2023</v>
       </c>
       <c r="K9" s="20"/>
       <c r="L9" s="20"/>
       <c r="M9" s="20"/>
       <c r="N9" s="20"/>
-      <c r="P9" s="101">
+      <c r="P9" s="3">
         <f t="shared" si="3"/>
         <v>2023</v>
       </c>
@@ -39217,7 +39344,7 @@
         <f>$G$8</f>
         <v>1.0967771874057404</v>
       </c>
-      <c r="D10" s="101">
+      <c r="D10" s="3">
         <f t="shared" si="4"/>
         <v>2024</v>
       </c>
@@ -39225,14 +39352,14 @@
       <c r="F10" s="45"/>
       <c r="G10" s="45"/>
       <c r="H10" s="45"/>
-      <c r="J10" s="101">
+      <c r="J10" s="3">
         <v>2024</v>
       </c>
       <c r="K10" s="20"/>
       <c r="L10" s="20"/>
       <c r="M10" s="20"/>
       <c r="N10" s="20"/>
-      <c r="P10" s="101">
+      <c r="P10" s="3">
         <f t="shared" si="3"/>
         <v>2024</v>
       </c>
@@ -39248,6 +39375,12 @@
       <c r="B11" s="49">
         <f>$G$8</f>
         <v>1.0967771874057404</v>
+      </c>
+      <c r="K11" s="42" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q11" s="42" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
@@ -39293,7 +39426,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -39535,6 +39668,9 @@
         <f>$M$2</f>
         <v>0.62190000000000001</v>
       </c>
+      <c r="D4" s="107" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
@@ -39641,7 +39777,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -39651,7 +39787,7 @@
     <col min="1" max="1" width="9" style="2"/>
     <col min="2" max="2" width="10.7109375" style="2" customWidth="1"/>
     <col min="3" max="5" width="9" style="2"/>
-    <col min="6" max="6" width="9" style="7"/>
+    <col min="6" max="6" width="10.42578125" style="7" customWidth="1"/>
     <col min="7" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -39687,6 +39823,9 @@
       <c r="F2" s="67" t="s">
         <v>127</v>
       </c>
+      <c r="G2" s="42" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="68">
@@ -39780,7 +39919,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -40135,7 +40274,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <tabColor theme="0" tint="-0.499984740745262"/>
   </sheetPr>
@@ -40343,19 +40482,19 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="108">
+      <c r="A13" s="102">
         <v>46006</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J1" r:id="rId1"/>
-    <hyperlink ref="M1" r:id="rId2"/>
+    <hyperlink ref="J1" r:id="rId1" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
+    <hyperlink ref="M1" r:id="rId2" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>

</xml_diff>

<commit_message>
fetch fall enrollment and fte data from IPEDS
</commit_message>
<xml_diff>
--- a/_Source - CollegeControlTotal - 2025-02-14_Start.xlsx
+++ b/_Source - CollegeControlTotal - 2025-02-14_Start.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\TDM-INP-College-Enrollment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E45F1F1-8399-4D09-8170-582139454AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B23857BC-5F36-4059-9261-D3CCE4DB276E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="728" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="728" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export_ControlTot" sheetId="11" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="205">
   <si>
     <t>https://ushe.edu/institutional-data-resources-headcount/</t>
   </si>
@@ -684,6 +684,18 @@
   <si>
     <t>Project until 2060</t>
   </si>
+  <si>
+    <t>Brigham Young University</t>
+  </si>
+  <si>
+    <t>UofU</t>
+  </si>
+  <si>
+    <t>Salt Lake Community College</t>
+  </si>
+  <si>
+    <t>Ensign College</t>
+  </si>
 </sst>
 </file>
 
@@ -1014,7 +1026,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="2" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1276,6 +1288,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1285,14 +1305,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -22316,11 +22329,14 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="15" width="12.140625" style="7" customWidth="1"/>
-    <col min="16" max="21" width="9" style="7"/>
+    <col min="16" max="16" width="9" style="7"/>
+    <col min="17" max="17" width="12" style="7" customWidth="1"/>
+    <col min="18" max="18" width="29.42578125" style="7" customWidth="1"/>
+    <col min="19" max="21" width="9" style="7"/>
     <col min="22" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>112</v>
       </c>
@@ -22366,8 +22382,17 @@
       <c r="O1" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q1" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="110" t="s">
+        <v>201</v>
+      </c>
+      <c r="S1" s="7">
+        <v>230038</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1990</v>
       </c>
@@ -22427,8 +22452,17 @@
         <f>INDEX('Campus Enrol Disaggregation'!$P$5:$AC$65,MATCH(Export_ControlTot!$A2,'Campus Enrol Disaggregation'!$O$5:$O$65,0),MATCH(O$1,'Campus Enrol Disaggregation'!$P$4:$AC$4,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q2" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="R2" s="110" t="s">
+        <v>204</v>
+      </c>
+      <c r="S2" s="7">
+        <v>230418</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1991</v>
       </c>
@@ -22488,8 +22522,17 @@
         <f>INDEX('Campus Enrol Disaggregation'!$P$5:$AC$65,MATCH(Export_ControlTot!$A3,'Campus Enrol Disaggregation'!$O$5:$O$65,0),MATCH(O$1,'Campus Enrol Disaggregation'!$P$4:$AC$4,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q3" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="R3" s="110" t="s">
+        <v>203</v>
+      </c>
+      <c r="S3" s="7">
+        <v>230746</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>1992</v>
       </c>
@@ -22549,8 +22592,17 @@
         <f>INDEX('Campus Enrol Disaggregation'!$P$5:$AC$65,MATCH(Export_ControlTot!$A4,'Campus Enrol Disaggregation'!$O$5:$O$65,0),MATCH(O$1,'Campus Enrol Disaggregation'!$P$4:$AC$4,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q4" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="R4" s="110" t="s">
+        <v>142</v>
+      </c>
+      <c r="S4" s="7">
+        <v>230764</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>1993</v>
       </c>
@@ -22610,8 +22662,17 @@
         <f>INDEX('Campus Enrol Disaggregation'!$P$5:$AC$65,MATCH(Export_ControlTot!$A5,'Campus Enrol Disaggregation'!$O$5:$O$65,0),MATCH(O$1,'Campus Enrol Disaggregation'!$P$4:$AC$4,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q5" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="R5" s="110" t="s">
+        <v>140</v>
+      </c>
+      <c r="S5" s="7">
+        <v>230737</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>1994</v>
       </c>
@@ -22671,8 +22732,17 @@
         <f>INDEX('Campus Enrol Disaggregation'!$P$5:$AC$65,MATCH(Export_ControlTot!$A6,'Campus Enrol Disaggregation'!$O$5:$O$65,0),MATCH(O$1,'Campus Enrol Disaggregation'!$P$4:$AC$4,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q6" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="R6" s="110" t="s">
+        <v>143</v>
+      </c>
+      <c r="S6" s="7">
+        <v>230782</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>1995</v>
       </c>
@@ -22732,8 +22802,17 @@
         <f>INDEX('Campus Enrol Disaggregation'!$P$5:$AC$65,MATCH(Export_ControlTot!$A7,'Campus Enrol Disaggregation'!$O$5:$O$65,0),MATCH(O$1,'Campus Enrol Disaggregation'!$P$4:$AC$4,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="Q7" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="R7" s="110" t="s">
+        <v>146</v>
+      </c>
+      <c r="S7" s="7">
+        <v>230807</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>1996</v>
       </c>
@@ -22794,7 +22873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>1997</v>
       </c>
@@ -22855,7 +22934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>1998</v>
       </c>
@@ -22916,7 +22995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>1999</v>
       </c>
@@ -22977,7 +23056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>2000</v>
       </c>
@@ -23038,7 +23117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>2001</v>
       </c>
@@ -23099,7 +23178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>2002</v>
       </c>
@@ -23160,7 +23239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>2003</v>
       </c>
@@ -23221,7 +23300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>2004</v>
       </c>
@@ -26117,7 +26196,7 @@
       <c r="A68" s="7">
         <v>2056</v>
       </c>
-      <c r="B68" s="108"/>
+      <c r="B68" s="105"/>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="7">
@@ -26140,7 +26219,7 @@
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="109" t="s">
+      <c r="A73" s="106" t="s">
         <v>198</v>
       </c>
     </row>
@@ -26177,30 +26256,30 @@
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="J2" s="5"/>
-      <c r="Q2" s="103" t="s">
+      <c r="Q2" s="107" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="104"/>
-      <c r="S2" s="104"/>
-      <c r="T2" s="104"/>
-      <c r="U2" s="103" t="s">
+      <c r="R2" s="108"/>
+      <c r="S2" s="108"/>
+      <c r="T2" s="108"/>
+      <c r="U2" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="104"/>
-      <c r="W2" s="104"/>
-      <c r="X2" s="104"/>
-      <c r="Y2" s="103" t="s">
+      <c r="V2" s="108"/>
+      <c r="W2" s="108"/>
+      <c r="X2" s="108"/>
+      <c r="Y2" s="107" t="s">
         <v>3</v>
       </c>
-      <c r="Z2" s="104"/>
-      <c r="AA2" s="104"/>
-      <c r="AB2" s="104"/>
-      <c r="AC2" s="103" t="s">
+      <c r="Z2" s="108"/>
+      <c r="AA2" s="108"/>
+      <c r="AB2" s="108"/>
+      <c r="AC2" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="AD2" s="104"/>
-      <c r="AE2" s="104"/>
-      <c r="AF2" s="104"/>
+      <c r="AD2" s="108"/>
+      <c r="AE2" s="108"/>
+      <c r="AF2" s="108"/>
     </row>
     <row r="3" spans="1:32" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -28004,7 +28083,7 @@
       <c r="A8" s="2">
         <v>2020</v>
       </c>
-      <c r="B8" s="106">
+      <c r="B8" s="103">
         <f>AVERAGE(B7,B9)</f>
         <v>1830</v>
       </c>
@@ -30004,196 +30083,196 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="105" t="s">
+      <c r="B31" s="109" t="s">
         <v>46</v>
       </c>
-      <c r="C31" s="105"/>
-      <c r="D31" s="105"/>
-      <c r="E31" s="105"/>
+      <c r="C31" s="109"/>
+      <c r="D31" s="109"/>
+      <c r="E31" s="109"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B32" s="105"/>
-      <c r="C32" s="105"/>
-      <c r="D32" s="105"/>
-      <c r="E32" s="105"/>
+      <c r="B32" s="109"/>
+      <c r="C32" s="109"/>
+      <c r="D32" s="109"/>
+      <c r="E32" s="109"/>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" s="105"/>
-      <c r="C33" s="105"/>
-      <c r="D33" s="105"/>
-      <c r="E33" s="105"/>
+      <c r="B33" s="109"/>
+      <c r="C33" s="109"/>
+      <c r="D33" s="109"/>
+      <c r="E33" s="109"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" s="105"/>
-      <c r="C34" s="105"/>
-      <c r="D34" s="105"/>
-      <c r="E34" s="105"/>
+      <c r="B34" s="109"/>
+      <c r="C34" s="109"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="109"/>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" s="105"/>
-      <c r="C35" s="105"/>
-      <c r="D35" s="105"/>
-      <c r="E35" s="105"/>
+      <c r="B35" s="109"/>
+      <c r="C35" s="109"/>
+      <c r="D35" s="109"/>
+      <c r="E35" s="109"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B36" s="105"/>
-      <c r="C36" s="105"/>
-      <c r="D36" s="105"/>
-      <c r="E36" s="105"/>
+      <c r="B36" s="109"/>
+      <c r="C36" s="109"/>
+      <c r="D36" s="109"/>
+      <c r="E36" s="109"/>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B37" s="105"/>
-      <c r="C37" s="105"/>
-      <c r="D37" s="105"/>
-      <c r="E37" s="105"/>
+      <c r="B37" s="109"/>
+      <c r="C37" s="109"/>
+      <c r="D37" s="109"/>
+      <c r="E37" s="109"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B38" s="105"/>
-      <c r="C38" s="105"/>
-      <c r="D38" s="105"/>
-      <c r="E38" s="105"/>
+      <c r="B38" s="109"/>
+      <c r="C38" s="109"/>
+      <c r="D38" s="109"/>
+      <c r="E38" s="109"/>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B39" s="105"/>
-      <c r="C39" s="105"/>
-      <c r="D39" s="105"/>
-      <c r="E39" s="105"/>
+      <c r="B39" s="109"/>
+      <c r="C39" s="109"/>
+      <c r="D39" s="109"/>
+      <c r="E39" s="109"/>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B40" s="105"/>
-      <c r="C40" s="105"/>
-      <c r="D40" s="105"/>
-      <c r="E40" s="105"/>
+      <c r="B40" s="109"/>
+      <c r="C40" s="109"/>
+      <c r="D40" s="109"/>
+      <c r="E40" s="109"/>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B41" s="105"/>
-      <c r="C41" s="105"/>
-      <c r="D41" s="105"/>
-      <c r="E41" s="105"/>
+      <c r="B41" s="109"/>
+      <c r="C41" s="109"/>
+      <c r="D41" s="109"/>
+      <c r="E41" s="109"/>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B42" s="105"/>
-      <c r="C42" s="105"/>
-      <c r="D42" s="105"/>
-      <c r="E42" s="105"/>
+      <c r="B42" s="109"/>
+      <c r="C42" s="109"/>
+      <c r="D42" s="109"/>
+      <c r="E42" s="109"/>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B43" s="105"/>
-      <c r="C43" s="105"/>
-      <c r="D43" s="105"/>
-      <c r="E43" s="105"/>
+      <c r="B43" s="109"/>
+      <c r="C43" s="109"/>
+      <c r="D43" s="109"/>
+      <c r="E43" s="109"/>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B44" s="105"/>
-      <c r="C44" s="105"/>
-      <c r="D44" s="105"/>
-      <c r="E44" s="105"/>
+      <c r="B44" s="109"/>
+      <c r="C44" s="109"/>
+      <c r="D44" s="109"/>
+      <c r="E44" s="109"/>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B46" s="105" t="s">
+      <c r="B46" s="109" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="105"/>
-      <c r="D46" s="105"/>
-      <c r="E46" s="105"/>
+      <c r="C46" s="109"/>
+      <c r="D46" s="109"/>
+      <c r="E46" s="109"/>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B47" s="105" t="s">
+      <c r="B47" s="109" t="s">
         <v>45</v>
       </c>
-      <c r="C47" s="105"/>
-      <c r="D47" s="105"/>
-      <c r="E47" s="105"/>
+      <c r="C47" s="109"/>
+      <c r="D47" s="109"/>
+      <c r="E47" s="109"/>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B48" s="105"/>
-      <c r="C48" s="105"/>
-      <c r="D48" s="105"/>
-      <c r="E48" s="105"/>
+      <c r="B48" s="109"/>
+      <c r="C48" s="109"/>
+      <c r="D48" s="109"/>
+      <c r="E48" s="109"/>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B49" s="105"/>
-      <c r="C49" s="105"/>
-      <c r="D49" s="105"/>
-      <c r="E49" s="105"/>
+      <c r="B49" s="109"/>
+      <c r="C49" s="109"/>
+      <c r="D49" s="109"/>
+      <c r="E49" s="109"/>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B50" s="105"/>
-      <c r="C50" s="105"/>
-      <c r="D50" s="105"/>
-      <c r="E50" s="105"/>
+      <c r="B50" s="109"/>
+      <c r="C50" s="109"/>
+      <c r="D50" s="109"/>
+      <c r="E50" s="109"/>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B51" s="105"/>
-      <c r="C51" s="105"/>
-      <c r="D51" s="105"/>
-      <c r="E51" s="105"/>
+      <c r="B51" s="109"/>
+      <c r="C51" s="109"/>
+      <c r="D51" s="109"/>
+      <c r="E51" s="109"/>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B52" s="105"/>
-      <c r="C52" s="105"/>
-      <c r="D52" s="105"/>
-      <c r="E52" s="105"/>
+      <c r="B52" s="109"/>
+      <c r="C52" s="109"/>
+      <c r="D52" s="109"/>
+      <c r="E52" s="109"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B53" s="105"/>
-      <c r="C53" s="105"/>
-      <c r="D53" s="105"/>
-      <c r="E53" s="105"/>
+      <c r="B53" s="109"/>
+      <c r="C53" s="109"/>
+      <c r="D53" s="109"/>
+      <c r="E53" s="109"/>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B54" s="105"/>
-      <c r="C54" s="105"/>
-      <c r="D54" s="105"/>
-      <c r="E54" s="105"/>
+      <c r="B54" s="109"/>
+      <c r="C54" s="109"/>
+      <c r="D54" s="109"/>
+      <c r="E54" s="109"/>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B55" s="105"/>
-      <c r="C55" s="105"/>
-      <c r="D55" s="105"/>
-      <c r="E55" s="105"/>
+      <c r="B55" s="109"/>
+      <c r="C55" s="109"/>
+      <c r="D55" s="109"/>
+      <c r="E55" s="109"/>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B56" s="105"/>
-      <c r="C56" s="105"/>
-      <c r="D56" s="105"/>
-      <c r="E56" s="105"/>
+      <c r="B56" s="109"/>
+      <c r="C56" s="109"/>
+      <c r="D56" s="109"/>
+      <c r="E56" s="109"/>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B57" s="105"/>
-      <c r="C57" s="105"/>
-      <c r="D57" s="105"/>
-      <c r="E57" s="105"/>
+      <c r="B57" s="109"/>
+      <c r="C57" s="109"/>
+      <c r="D57" s="109"/>
+      <c r="E57" s="109"/>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B58" s="105"/>
-      <c r="C58" s="105"/>
-      <c r="D58" s="105"/>
-      <c r="E58" s="105"/>
+      <c r="B58" s="109"/>
+      <c r="C58" s="109"/>
+      <c r="D58" s="109"/>
+      <c r="E58" s="109"/>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B59" s="105"/>
-      <c r="C59" s="105"/>
-      <c r="D59" s="105"/>
-      <c r="E59" s="105"/>
+      <c r="B59" s="109"/>
+      <c r="C59" s="109"/>
+      <c r="D59" s="109"/>
+      <c r="E59" s="109"/>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B60" s="105"/>
-      <c r="C60" s="105"/>
-      <c r="D60" s="105"/>
-      <c r="E60" s="105"/>
+      <c r="B60" s="109"/>
+      <c r="C60" s="109"/>
+      <c r="D60" s="109"/>
+      <c r="E60" s="109"/>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B61" s="105"/>
-      <c r="C61" s="105"/>
-      <c r="D61" s="105"/>
-      <c r="E61" s="105"/>
+      <c r="B61" s="109"/>
+      <c r="C61" s="109"/>
+      <c r="D61" s="109"/>
+      <c r="E61" s="109"/>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B62" s="105"/>
-      <c r="C62" s="105"/>
-      <c r="D62" s="105"/>
-      <c r="E62" s="105"/>
+      <c r="B62" s="109"/>
+      <c r="C62" s="109"/>
+      <c r="D62" s="109"/>
+      <c r="E62" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -36427,7 +36506,7 @@
       </c>
     </row>
     <row r="66" spans="15:30" x14ac:dyDescent="0.25">
-      <c r="O66" s="108" t="s">
+      <c r="O66" s="105" t="s">
         <v>199</v>
       </c>
     </row>
@@ -38828,7 +38907,7 @@
       </c>
     </row>
     <row r="65" spans="35:35" x14ac:dyDescent="0.25">
-      <c r="AI65" s="108" t="s">
+      <c r="AI65" s="105" t="s">
         <v>200</v>
       </c>
     </row>
@@ -39668,7 +39747,7 @@
         <f>$M$2</f>
         <v>0.62190000000000001</v>
       </c>
-      <c r="D4" s="107" t="s">
+      <c r="D4" s="104" t="s">
         <v>196</v>
       </c>
     </row>

</xml_diff>